<commit_message>
docs: apply review fixes to business strategy and model
- Show all-in per-user pricing (hardware + setup) alongside the
  subscription-only figure and soften comparisons with cloud tools
- Reserve "air-gapped" for strict mode; reword offline claims elsewhere
- Soften privilege/consent claims to match what Heppner and ABA 512 say
- Resequence the 90-day plan and roadmap so marketing shows only shipped
  features, accuracy is measured before pilots, and CPA/defense tracks
  have explicit go/no-go gates
- Require hardware paid in full on order; align design-partner terms
- Add reseller-channel inputs to the model (default 0%) and document the
  30%-resold sensitivity; correct referral-fee economics
- Fix unsourced competitor claims, lead-time and deposit contradictions,
  build-warning and parse-failure descriptions, and the diagram borders

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDEQCSX5jr3s79EPtgeMEg
</commit_message>
<xml_diff>
--- a/docs/business/financial-model.xlsx
+++ b/docs/business/financial-model.xlsx
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="378">
   <si>
     <t xml:space="preserve">Private AI Appliance - Pricing &amp; Unit Economics Model</t>
   </si>
@@ -164,6 +164,9 @@
     <t xml:space="preserve">- Hires start automatically the month after total active clients reach each role's threshold (Opex Plan), so weaker sales delay hiring. Founder pay and other opex are fixed by year.</t>
   </si>
   <si>
+    <t xml:space="preserve">- Partner channel: Assumptions!B31-B32 apply a reseller discount to that share of subscription revenue (default 0% = every client pays list). Referral fees and partner-handled support are not modeled.</t>
+  </si>
+  <si>
     <t xml:space="preserve">- Excludes income taxes, sales tax on hardware (collected and remitted, not revenue), and financing costs.</t>
   </si>
   <si>
@@ -239,10 +242,10 @@
     <t xml:space="preserve">Negative = funding required</t>
   </si>
   <si>
-    <t xml:space="preserve">ARR at year end (list price)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annual recurring revenue run-rate</t>
+    <t xml:space="preserve">ARR at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subscription run-rate x 12, after any partner discounts</t>
   </si>
   <si>
     <t xml:space="preserve">Hires on payroll at year end (excl. founders)</t>
@@ -488,7 +491,7 @@
     <t xml:space="preserve">Hardware markup over cost (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cost-plus pass-through. Benchmarks: channel hardware markup 20-28% and shrinking; CDW 21.7% gross margin FY2025; Datto sold appliances below cost to win subscriptions. Keep it thin: buyers can price-check a DGX Spark.</t>
+    <t xml:space="preserve">Cost-plus pass-through, paid in full on order. Benchmarks: channel hardware markup 20-28% and shrinking; CDW 21.7% gross margin FY2025; Datto sold appliances below cost to win subscriptions. Keep it thin: buyers can price-check a DGX Spark.</t>
   </si>
   <si>
     <t xml:space="preserve">Hardware cost to us ($)</t>
@@ -587,6 +590,18 @@
     <t xml:space="preserve">Caps LTV so low churn doesn't imply an unrealistic lifetime.</t>
   </si>
   <si>
+    <t xml:space="preserve">Share of clients sold through reseller partners (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set above 0% to model MSP resale. The go-to-market plan targets ~30% of pipeline from MSPs (referral + resale). Default 0% = every client pays list.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reseller discount on subscription (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical reseller discount on the subscription is 20-30% (05-go-to-market.md).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sales Plan: new clients signed per quarter</t>
   </si>
   <si>
@@ -698,7 +713,7 @@
     <t xml:space="preserve">Marketing, events and CLE</t>
   </si>
   <si>
-    <t xml:space="preserve">Year 1: ABA TECHSHOW 10x10 booth $5,050 + furniture $1,855 (Mar 2027), CLE accreditation fees (CA $159/activity; IL $50/course + $0.75/attorney-hour), local association sponsorships, content. Later: AICPA ENGAGE booth $6,800, state association booths ~$1.5-2k, Legalweek.</t>
+    <t xml:space="preserve">Year 1: attend ABA TECHSHOW (Mar 2027) as a visitor, or exhibit only if you have 3+ references by then (10x10 booth $5,050 + furniture $1,855); CLE accreditation fees (CA $159/activity; IL $50/course + $0.75/attorney-hour); local association sponsorships; content. Later years: booths such as AICPA ENGAGE ($6,800) and state associations (~$1.5-2k); Legalweek vendor pass ($4,995).</t>
   </si>
   <si>
     <t xml:space="preserve">Sales travel</t>
@@ -845,7 +860,7 @@
     <t xml:space="preserve">Cash balance (end of month)</t>
   </si>
   <si>
-    <t xml:space="preserve">ARR at list price (subscriptions x 12)</t>
+    <t xml:space="preserve">ARR (subscriptions x 12, after partner discounts, before design-partner discount)</t>
   </si>
   <si>
     <t xml:space="preserve">Helper: month number if EBITDA &gt;= 0 from here through month 36, else 999</t>
@@ -1772,7 +1787,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1885,6 +1900,11 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1913,7 +1933,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1924,24 +1944,24 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$7:$AK$7)+SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$8:$AK$8)+SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$9:$AK$9)</f>
@@ -1956,12 +1976,12 @@
         <v>30</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">INDEX(Projection!$B$15:$AK$15,1,12*1)</f>
@@ -1979,12 +1999,12 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$18:$AK$18)</f>
@@ -1999,12 +2019,12 @@
         <v>641790.85</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$19:$AK$19)</f>
@@ -2022,7 +2042,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$20:$AK$20)</f>
@@ -2037,12 +2057,12 @@
         <v>1245644.98038372</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">SUM(B8:B10)</f>
@@ -2060,7 +2080,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$28:$AK$28)</f>
@@ -2078,7 +2098,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">IF(B11=0,0,B12/B11)</f>
@@ -2096,7 +2116,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$40:$AK$40)</f>
@@ -2114,7 +2134,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">B12-B14</f>
@@ -2132,7 +2152,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$43:$AK$43)</f>
@@ -2150,7 +2170,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$45:$AK$45,1,12*1)</f>
@@ -2165,12 +2185,12 @@
         <v>65489.5340109068</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$47:$AK$47,1,12*1)</f>
@@ -2185,12 +2205,12 @@
         <v>1780192.88340635</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" s="14" t="n">
         <f aca="false">Projection!$M$49+Projection!$M$50+Projection!$M$51+Projection!$M$52</f>
@@ -2205,17 +2225,17 @@
         <v>4</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" s="15" t="n">
         <f aca="false">IF(MIN(Projection!$B$48:$AK$48)=999,"Not within 36 months",MIN(Projection!$B$48:$AK$48))</f>
@@ -2224,7 +2244,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">MIN(Projection!$B$45:$AK$45)</f>
@@ -2233,19 +2253,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B23" s="16" t="n">
         <f aca="false">MAX(0,-B22)</f>
         <v>286825.263119692</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">Projection!$AK$15</f>
@@ -2254,25 +2274,25 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B28" s="14" t="n">
         <f aca="false">IFERROR(MATCH(1,Projection!$B$49:$AK$49,0),"Not within 36 months")</f>
@@ -2285,7 +2305,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B29" s="14" t="n">
         <f aca="false">IFERROR(MATCH(1,Projection!$B$50:$AK$50,0),"Not within 36 months")</f>
@@ -2298,7 +2318,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B30" s="14" t="n">
         <f aca="false">IFERROR(MATCH(1,Projection!$B$51:$AK$51,0),"Not within 36 months")</f>
@@ -2311,7 +2331,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B31" s="14" t="n">
         <f aca="false">IFERROR(MATCH(1,Projection!$B$52:$AK$52,0),"Not within 36 months")</f>
@@ -2348,34 +2368,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">Assumptions!B20*Assumptions!$B$5</f>
@@ -2390,12 +2410,12 @@
         <v>66700</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">Assumptions!B11</f>
@@ -2413,7 +2433,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">B5+B6</f>
@@ -2431,7 +2451,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">Assumptions!B14*Assumptions!$B$5</f>
@@ -2449,7 +2469,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">Assumptions!B15*Assumptions!$B$23+Assumptions!B16</f>
@@ -2464,12 +2484,12 @@
         <v>11500</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">B7-B8-B9</f>
@@ -2487,7 +2507,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">IF(B7=0,0,B10/B7)</f>
@@ -2505,12 +2525,12 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">Assumptions!B12</f>
@@ -2528,7 +2548,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B14" s="17" t="n">
         <f aca="false">Assumptions!B17*Assumptions!$B$23+Assumptions!B18</f>
@@ -2543,12 +2563,12 @@
         <v>1330</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">B13-B14</f>
@@ -2566,7 +2586,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B16" s="13" t="n">
         <f aca="false">IF(B13=0,0,B15/B13)</f>
@@ -2584,7 +2604,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IF(Assumptions!B10=0,0,B13/Assumptions!B10)</f>
@@ -2599,17 +2619,17 @@
         <v>56.6666666666667</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">B7+12*B13</f>
@@ -2624,12 +2644,12 @@
         <v>193700</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B20" s="12" t="n">
         <f aca="false">B10+12*B15</f>
@@ -2647,7 +2667,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B21" s="13" t="n">
         <f aca="false">IF(B19=0,0,B20/B19)</f>
@@ -2662,12 +2682,12 @@
         <v>0.55880227155395</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B22" s="17" t="n">
         <f aca="false">12*B13</f>
@@ -2685,7 +2705,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B23" s="17" t="n">
         <f aca="false">12*B15</f>
@@ -2703,12 +2723,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">MIN(Assumptions!$B$30,IF(Assumptions!$B$24=0,Assumptions!$B$30,1/Assumptions!$B$24))</f>
@@ -2723,12 +2743,12 @@
         <v>5</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">B10+B23*B25</f>
@@ -2743,12 +2763,12 @@
         <v>452400</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B27" s="17" t="n">
         <f aca="false">Assumptions!B19</f>
@@ -2766,7 +2786,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B28" s="19" t="n">
         <f aca="false">IF(B27=0,0,B26/B27)</f>
@@ -2781,12 +2801,12 @@
         <v>18.096</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">IF(B15&lt;=0,0,MAX(0,B27-B10)/B15)</f>
@@ -2801,17 +2821,17 @@
         <v>0.390516039051604</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B31" s="20" t="n">
         <f aca="false">Assumptions!B15+12*Assumptions!B17</f>
@@ -2826,12 +2846,12 @@
         <v>244</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B32" s="20" t="n">
         <f aca="false">IF(Assumptions!B17=0,0,Assumptions!$B$29/(12*Assumptions!B17))</f>
@@ -2846,7 +2866,7 @@
         <v>9.72222222222222</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2865,7 +2885,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -2875,17 +2895,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B4" s="21" t="n">
         <v>2</v>
@@ -2893,7 +2913,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>1</v>
@@ -2901,7 +2921,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B6" s="22" t="n">
         <v>0</v>
@@ -2909,41 +2929,41 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B10" s="23" t="n">
         <v>12</v>
@@ -2955,12 +2975,12 @@
         <v>150</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>4500</v>
@@ -2972,12 +2992,12 @@
         <v>25000</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B12" s="22" t="n">
         <v>1500</v>
@@ -2989,12 +3009,12 @@
         <v>8500</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B13" s="24" t="n">
         <v>0.15</v>
@@ -3006,12 +3026,12 @@
         <v>0.15</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B14" s="11" t="n">
         <f aca="false">'Hardware BOM'!$D$10</f>
@@ -3026,12 +3046,12 @@
         <v>58000</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B15" s="23" t="n">
         <v>20</v>
@@ -3043,12 +3063,12 @@
         <v>100</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B16" s="25" t="n">
         <v>400</v>
@@ -3060,12 +3080,12 @@
         <v>2500</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B17" s="26" t="n">
         <v>2.5</v>
@@ -3077,12 +3097,12 @@
         <v>12</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B18" s="25" t="n">
         <v>50</v>
@@ -3094,12 +3114,12 @@
         <v>250</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B19" s="22" t="n">
         <v>6000</v>
@@ -3111,12 +3131,12 @@
         <v>25000</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">B14*(1+B13)</f>
@@ -3131,109 +3151,131 @@
         <v>66700</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B23" s="22" t="n">
         <v>90</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B24" s="24" t="n">
         <v>0.1</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B25" s="27" t="n">
         <f aca="false">1-(1-B24)^(1/12)</f>
         <v>0.00874161095469672</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B26" s="24" t="n">
         <v>0.3</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B27" s="28" t="n">
         <v>0.2</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B28" s="28" t="n">
         <v>0.1</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B29" s="23" t="n">
         <v>1400</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B30" s="23" t="n">
         <v>5</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B32" s="28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -3264,67 +3306,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C5" s="23" t="n">
         <v>0</v>
@@ -3367,15 +3409,15 @@
         <v>15</v>
       </c>
       <c r="P5" s="29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>0</v>
@@ -3421,10 +3463,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>0</v>
@@ -3470,10 +3512,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>0</v>
@@ -3519,10 +3561,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>0</v>
@@ -3568,10 +3610,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>0</v>
@@ -3617,10 +3659,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>0</v>
@@ -3666,10 +3708,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>0</v>
@@ -3715,10 +3757,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>0</v>
@@ -3764,7 +3806,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B15" s="30"/>
       <c r="C15" s="30"/>
@@ -3783,10 +3825,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C16" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,C5,C8,C11)</f>
@@ -3843,10 +3885,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,C6,C9,C12)</f>
@@ -3903,10 +3945,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C18" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,C7,C10,C13)</f>
@@ -3990,34 +4032,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B4" s="25" t="n">
         <v>72000</v>
@@ -4029,12 +4071,12 @@
         <v>264000</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B5" s="25" t="n">
         <v>10000</v>
@@ -4046,12 +4088,12 @@
         <v>30000</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B6" s="25" t="n">
         <v>4000</v>
@@ -4063,12 +4105,12 @@
         <v>14000</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B7" s="25" t="n">
         <v>15000</v>
@@ -4080,12 +4122,12 @@
         <v>20000</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B8" s="25" t="n">
         <v>9000</v>
@@ -4097,12 +4139,12 @@
         <v>45000</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="B9" s="25" t="n">
         <v>15000</v>
@@ -4114,12 +4156,12 @@
         <v>70000</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B10" s="25" t="n">
         <v>12000</v>
@@ -4131,27 +4173,27 @@
         <v>36000</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="25" t="n">
         <v>105000</v>
@@ -4160,12 +4202,12 @@
         <v>5</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B14" s="25" t="n">
         <v>85000</v>
@@ -4174,12 +4216,12 @@
         <v>8</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="25" t="n">
         <v>115000</v>
@@ -4188,12 +4230,12 @@
         <v>25</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B16" s="25" t="n">
         <v>75000</v>
@@ -4202,27 +4244,27 @@
         <v>40</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B19" s="25" t="n">
         <v>5500</v>
@@ -4231,12 +4273,12 @@
         <v>1</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="B20" s="25" t="n">
         <v>22500</v>
@@ -4245,12 +4287,12 @@
         <v>5</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B21" s="25" t="n">
         <v>8000</v>
@@ -4259,7 +4301,7 @@
         <v>13</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -4288,12 +4330,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B2" s="31" t="n">
         <v>1</v>
@@ -4406,7 +4448,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B3" s="20" t="n">
         <f aca="false">ROUNDUP(B2/12,0)</f>
@@ -4555,7 +4597,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B4" s="20" t="n">
         <f aca="false">ROUNDUP(B2/3,0)</f>
@@ -4704,12 +4746,12 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,B$4)/3</f>
@@ -4858,7 +4900,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,B$4)/3</f>
@@ -5007,7 +5049,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$18:$N$18,1,B$4)/3</f>
@@ -5156,12 +5198,12 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B12" s="18" t="n">
         <f aca="false">B7</f>
@@ -5310,7 +5352,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B13" s="18" t="n">
         <f aca="false">B8</f>
@@ -5459,7 +5501,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B14" s="18" t="n">
         <f aca="false">B9</f>
@@ -5608,7 +5650,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">SUM(B12:B14)</f>
@@ -5757,12 +5799,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">(B7*Assumptions!$B$20+B8*Assumptions!$C$20+B9*Assumptions!$D$20)*Assumptions!$B$5</f>
@@ -5911,7 +5953,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">B7*Assumptions!$B$11+B8*Assumptions!$C$11+B9*Assumptions!$D$11</f>
@@ -6060,156 +6102,156 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B20" s="17" t="n">
-        <f aca="false">(B12*Assumptions!$B$12+B13*Assumptions!$C$12+B14*Assumptions!$D$12)*(1-IF(B$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(B12*Assumptions!$B$12+B13*Assumptions!$C$12+B14*Assumptions!$D$12)*(1-IF(B$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>0</v>
       </c>
       <c r="C20" s="17" t="n">
-        <f aca="false">(C12*Assumptions!$B$12+C13*Assumptions!$C$12+C14*Assumptions!$D$12)*(1-IF(C$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(C12*Assumptions!$B$12+C13*Assumptions!$C$12+C14*Assumptions!$D$12)*(1-IF(C$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>0</v>
       </c>
       <c r="D20" s="17" t="n">
-        <f aca="false">(D12*Assumptions!$B$12+D13*Assumptions!$C$12+D14*Assumptions!$D$12)*(1-IF(D$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(D12*Assumptions!$B$12+D13*Assumptions!$C$12+D14*Assumptions!$D$12)*(1-IF(D$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>0</v>
       </c>
       <c r="E20" s="17" t="n">
-        <f aca="false">(E12*Assumptions!$B$12+E13*Assumptions!$C$12+E14*Assumptions!$D$12)*(1-IF(E$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(E12*Assumptions!$B$12+E13*Assumptions!$C$12+E14*Assumptions!$D$12)*(1-IF(E$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>350</v>
       </c>
       <c r="F20" s="17" t="n">
-        <f aca="false">(F12*Assumptions!$B$12+F13*Assumptions!$C$12+F14*Assumptions!$D$12)*(1-IF(F$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(F12*Assumptions!$B$12+F13*Assumptions!$C$12+F14*Assumptions!$D$12)*(1-IF(F$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>696.940436165856</v>
       </c>
       <c r="G20" s="17" t="n">
-        <f aca="false">(G12*Assumptions!$B$12+G13*Assumptions!$C$12+G14*Assumptions!$D$12)*(1-IF(G$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(G12*Assumptions!$B$12+G13*Assumptions!$C$12+G14*Assumptions!$D$12)*(1-IF(G$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1040.8480540143</v>
       </c>
       <c r="H20" s="17" t="n">
-        <f aca="false">(H12*Assumptions!$B$12+H13*Assumptions!$C$12+H14*Assumptions!$D$12)*(1-IF(H$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(H12*Assumptions!$B$12+H13*Assumptions!$C$12+H14*Assumptions!$D$12)*(1-IF(H$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>2315.08269859648</v>
       </c>
       <c r="I20" s="17" t="n">
-        <f aca="false">(I12*Assumptions!$B$12+I13*Assumptions!$C$12+I14*Assumptions!$D$12)*(1-IF(I$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(I12*Assumptions!$B$12+I13*Assumptions!$C$12+I14*Assumptions!$D$12)*(1-IF(I$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>3578.17847965074</v>
       </c>
       <c r="J20" s="17" t="n">
-        <f aca="false">(J12*Assumptions!$B$12+J13*Assumptions!$C$12+J14*Assumptions!$D$12)*(1-IF(J$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(J12*Assumptions!$B$12+J13*Assumptions!$C$12+J14*Assumptions!$D$12)*(1-IF(J$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>4830.2327687885</v>
       </c>
       <c r="K20" s="17" t="n">
-        <f aca="false">(K12*Assumptions!$B$12+K13*Assumptions!$C$12+K14*Assumptions!$D$12)*(1-IF(K$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(K12*Assumptions!$B$12+K13*Assumptions!$C$12+K14*Assumptions!$D$12)*(1-IF(K$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>6071.34208643645</v>
       </c>
       <c r="L20" s="17" t="n">
-        <f aca="false">(L12*Assumptions!$B$12+L13*Assumptions!$C$12+L14*Assumptions!$D$12)*(1-IF(L$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(L12*Assumptions!$B$12+L13*Assumptions!$C$12+L14*Assumptions!$D$12)*(1-IF(L$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>7301.60210927728</v>
       </c>
       <c r="M20" s="17" t="n">
-        <f aca="false">(M12*Assumptions!$B$12+M13*Assumptions!$C$12+M14*Assumptions!$D$12)*(1-IF(M$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(M12*Assumptions!$B$12+M13*Assumptions!$C$12+M14*Assumptions!$D$12)*(1-IF(M$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>8521.10767762532</v>
       </c>
       <c r="N20" s="17" t="n">
-        <f aca="false">(N12*Assumptions!$B$12+N13*Assumptions!$C$12+N14*Assumptions!$D$12)*(1-IF(N$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(N12*Assumptions!$B$12+N13*Assumptions!$C$12+N14*Assumptions!$D$12)*(1-IF(N$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>14399.9325753397</v>
       </c>
       <c r="O20" s="17" t="n">
-        <f aca="false">(O12*Assumptions!$B$12+O13*Assumptions!$C$12+O14*Assumptions!$D$12)*(1-IF(O$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(O12*Assumptions!$B$12+O13*Assumptions!$C$12+O14*Assumptions!$D$12)*(1-IF(O$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>16607.3873003255</v>
       </c>
       <c r="P20" s="17" t="n">
-        <f aca="false">(P12*Assumptions!$B$12+P13*Assumptions!$C$12+P14*Assumptions!$D$12)*(1-IF(P$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(P12*Assumptions!$B$12+P13*Assumptions!$C$12+P14*Assumptions!$D$12)*(1-IF(P$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>18795.5453149054</v>
       </c>
       <c r="Q20" s="17" t="n">
-        <f aca="false">(Q12*Assumptions!$B$12+Q13*Assumptions!$C$12+Q14*Assumptions!$D$12)*(1-IF(Q$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(Q12*Assumptions!$B$12+Q13*Assumptions!$C$12+Q14*Assumptions!$D$12)*(1-IF(Q$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>22297.9086367478</v>
       </c>
       <c r="R20" s="17" t="n">
-        <f aca="false">(R12*Assumptions!$B$12+R13*Assumptions!$C$12+R14*Assumptions!$D$12)*(1-IF(R$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(R12*Assumptions!$B$12+R13*Assumptions!$C$12+R14*Assumptions!$D$12)*(1-IF(R$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>25769.6556610087</v>
       </c>
       <c r="S20" s="17" t="n">
-        <f aca="false">(S12*Assumptions!$B$12+S13*Assumptions!$C$12+S14*Assumptions!$D$12)*(1-IF(S$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(S12*Assumptions!$B$12+S13*Assumptions!$C$12+S14*Assumptions!$D$12)*(1-IF(S$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>29211.0540234503</v>
       </c>
       <c r="T20" s="17" t="n">
-        <f aca="false">(T12*Assumptions!$B$12+T13*Assumptions!$C$12+T14*Assumptions!$D$12)*(1-IF(T$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(T12*Assumptions!$B$12+T13*Assumptions!$C$12+T14*Assumptions!$D$12)*(1-IF(T$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>35455.7023536007</v>
       </c>
       <c r="U20" s="17" t="n">
-        <f aca="false">(U12*Assumptions!$B$12+U13*Assumptions!$C$12+U14*Assumptions!$D$12)*(1-IF(U$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(U12*Assumptions!$B$12+U13*Assumptions!$C$12+U14*Assumptions!$D$12)*(1-IF(U$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>41645.7623975</v>
       </c>
       <c r="V20" s="17" t="n">
-        <f aca="false">(V12*Assumptions!$B$12+V13*Assumptions!$C$12+V14*Assumptions!$D$12)*(1-IF(V$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(V12*Assumptions!$B$12+V13*Assumptions!$C$12+V14*Assumptions!$D$12)*(1-IF(V$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>47781.7113447093</v>
       </c>
       <c r="W20" s="17" t="n">
-        <f aca="false">(W12*Assumptions!$B$12+W13*Assumptions!$C$12+W14*Assumptions!$D$12)*(1-IF(W$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(W12*Assumptions!$B$12+W13*Assumptions!$C$12+W14*Assumptions!$D$12)*(1-IF(W$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>51030.6888800509</v>
       </c>
       <c r="X20" s="17" t="n">
-        <f aca="false">(X12*Assumptions!$B$12+X13*Assumptions!$C$12+X14*Assumptions!$D$12)*(1-IF(X$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(X12*Assumptions!$B$12+X13*Assumptions!$C$12+X14*Assumptions!$D$12)*(1-IF(X$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>54251.265117778</v>
       </c>
       <c r="Y20" s="17" t="n">
-        <f aca="false">(Y12*Assumptions!$B$12+Y13*Assumptions!$C$12+Y14*Assumptions!$D$12)*(1-IF(Y$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(Y12*Assumptions!$B$12+Y13*Assumptions!$C$12+Y14*Assumptions!$D$12)*(1-IF(Y$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>57443.6883309849</v>
       </c>
       <c r="Z20" s="17" t="n">
-        <f aca="false">(Z12*Assumptions!$B$12+Z13*Assumptions!$C$12+Z14*Assumptions!$D$12)*(1-IF(Z$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(Z12*Assumptions!$B$12+Z13*Assumptions!$C$12+Z14*Assumptions!$D$12)*(1-IF(Z$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>65274.871289126</v>
       </c>
       <c r="AA20" s="17" t="n">
-        <f aca="false">(AA12*Assumptions!$B$12+AA13*Assumptions!$C$12+AA14*Assumptions!$D$12)*(1-IF(AA$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AA12*Assumptions!$B$12+AA13*Assumptions!$C$12+AA14*Assumptions!$D$12)*(1-IF(AA$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>73037.5970925318</v>
       </c>
       <c r="AB20" s="17" t="n">
-        <f aca="false">(AB12*Assumptions!$B$12+AB13*Assumptions!$C$12+AB14*Assumptions!$D$12)*(1-IF(AB$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AB12*Assumptions!$B$12+AB13*Assumptions!$C$12+AB14*Assumptions!$D$12)*(1-IF(AB$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>80732.4641670164</v>
       </c>
       <c r="AC20" s="17" t="n">
-        <f aca="false">(AC12*Assumptions!$B$12+AC13*Assumptions!$C$12+AC14*Assumptions!$D$12)*(1-IF(AC$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AC12*Assumptions!$B$12+AC13*Assumptions!$C$12+AC14*Assumptions!$D$12)*(1-IF(AC$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>85526.7323738543</v>
       </c>
       <c r="AD20" s="17" t="n">
-        <f aca="false">(AD12*Assumptions!$B$12+AD13*Assumptions!$C$12+AD14*Assumptions!$D$12)*(1-IF(AD$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AD12*Assumptions!$B$12+AD13*Assumptions!$C$12+AD14*Assumptions!$D$12)*(1-IF(AD$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>90279.0909532156</v>
       </c>
       <c r="AE20" s="17" t="n">
-        <f aca="false">(AE12*Assumptions!$B$12+AE13*Assumptions!$C$12+AE14*Assumptions!$D$12)*(1-IF(AE$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AE12*Assumptions!$B$12+AE13*Assumptions!$C$12+AE14*Assumptions!$D$12)*(1-IF(AE$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>94989.9062627589</v>
       </c>
       <c r="AF20" s="17" t="n">
-        <f aca="false">(AF12*Assumptions!$B$12+AF13*Assumptions!$C$12+AF14*Assumptions!$D$12)*(1-IF(AF$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AF12*Assumptions!$B$12+AF13*Assumptions!$C$12+AF14*Assumptions!$D$12)*(1-IF(AF$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>103826.208124253</v>
       </c>
       <c r="AG20" s="17" t="n">
-        <f aca="false">(AG12*Assumptions!$B$12+AG13*Assumptions!$C$12+AG14*Assumptions!$D$12)*(1-IF(AG$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AG12*Assumptions!$B$12+AG13*Assumptions!$C$12+AG14*Assumptions!$D$12)*(1-IF(AG$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>112585.266472597</v>
       </c>
       <c r="AH20" s="17" t="n">
-        <f aca="false">(AH12*Assumptions!$B$12+AH13*Assumptions!$C$12+AH14*Assumptions!$D$12)*(1-IF(AH$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AH12*Assumptions!$B$12+AH13*Assumptions!$C$12+AH14*Assumptions!$D$12)*(1-IF(AH$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>121267.756540529</v>
       </c>
       <c r="AI20" s="17" t="n">
-        <f aca="false">(AI12*Assumptions!$B$12+AI13*Assumptions!$C$12+AI14*Assumptions!$D$12)*(1-IF(AI$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AI12*Assumptions!$B$12+AI13*Assumptions!$C$12+AI14*Assumptions!$D$12)*(1-IF(AI$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>130374.347658169</v>
       </c>
       <c r="AJ20" s="17" t="n">
-        <f aca="false">(AJ12*Assumptions!$B$12+AJ13*Assumptions!$C$12+AJ14*Assumptions!$D$12)*(1-IF(AJ$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AJ12*Assumptions!$B$12+AJ13*Assumptions!$C$12+AJ14*Assumptions!$D$12)*(1-IF(AJ$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>139401.332499136</v>
       </c>
       <c r="AK20" s="17" t="n">
-        <f aca="false">(AK12*Assumptions!$B$12+AK13*Assumptions!$C$12+AK14*Assumptions!$D$12)*(1-IF(AK$3=1,Assumptions!$B$26,0))</f>
+        <f aca="false">(AK12*Assumptions!$B$12+AK13*Assumptions!$C$12+AK14*Assumptions!$D$12)*(1-IF(AK$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>148349.406950529</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">SUM(B18:B20)</f>
@@ -6358,12 +6400,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B24" s="17" t="n">
         <f aca="false">(B7*Assumptions!$B$14+B8*Assumptions!$C$14+B9*Assumptions!$D$14)*Assumptions!$B$5</f>
@@ -6512,7 +6554,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B25" s="17" t="n">
         <f aca="false">B7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+B8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+B9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
@@ -6661,7 +6703,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">B12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+B13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+B14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
@@ -6810,7 +6852,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">SUM(B24:B26)</f>
@@ -6959,7 +7001,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">B21-B27</f>
@@ -7108,7 +7150,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B29" s="13" t="n">
         <f aca="false">IF(B21=0,0,B28/B21)</f>
@@ -7257,12 +7299,12 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B32" s="17" t="n">
         <f aca="false">(INDEX('Opex Plan'!$B$4:$D$4,1,B$3)/12+SUMPRODUCT(B49:B52,'Opex Plan'!$B$13:$B$16)/12)*(1+Assumptions!$B$27)</f>
@@ -7411,7 +7453,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">INDEX('Opex Plan'!$B$5:$D$5,1,B$3)/12</f>
@@ -7560,7 +7602,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">INDEX('Opex Plan'!$B$6:$D$6,1,B$3)/12</f>
@@ -7709,7 +7751,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">INDEX('Opex Plan'!$B$7:$D$7,1,B$3)/12</f>
@@ -7858,7 +7900,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B36" s="11" t="n">
         <f aca="false">INDEX('Opex Plan'!$B$8:$D$8,1,B$3)/12</f>
@@ -8007,7 +8049,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">INDEX('Opex Plan'!$B$9:$D$9,1,B$3)/12</f>
@@ -8156,7 +8198,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">INDEX('Opex Plan'!$B$10:$D$10,1,B$3)/12</f>
@@ -8305,7 +8347,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B39" s="17" t="n">
         <f aca="false">SUM(B32:B38)*Assumptions!$B$28</f>
@@ -8454,7 +8496,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B40" s="12" t="n">
         <f aca="false">SUM(B32:B39)</f>
@@ -8603,7 +8645,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B42" s="33" t="n">
         <f aca="false">B28-B40</f>
@@ -8752,7 +8794,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">SUMPRODUCT(('Opex Plan'!$C$19:$C$21=B$2)*'Opex Plan'!$B$19:$B$21)</f>
@@ -8901,7 +8943,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B44" s="17" t="n">
         <f aca="false">B42-B43</f>
@@ -9050,7 +9092,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B45" s="33" t="n">
         <f aca="false">Assumptions!$B$6+B44</f>
@@ -9199,156 +9241,156 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B47" s="17" t="n">
-        <f aca="false">(B12*Assumptions!$B$12+B13*Assumptions!$C$12+B14*Assumptions!$D$12)*12</f>
+        <f aca="false">(B12*Assumptions!$B$12+B13*Assumptions!$C$12+B14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>0</v>
       </c>
       <c r="C47" s="17" t="n">
-        <f aca="false">(C12*Assumptions!$B$12+C13*Assumptions!$C$12+C14*Assumptions!$D$12)*12</f>
+        <f aca="false">(C12*Assumptions!$B$12+C13*Assumptions!$C$12+C14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>0</v>
       </c>
       <c r="D47" s="17" t="n">
-        <f aca="false">(D12*Assumptions!$B$12+D13*Assumptions!$C$12+D14*Assumptions!$D$12)*12</f>
+        <f aca="false">(D12*Assumptions!$B$12+D13*Assumptions!$C$12+D14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>0</v>
       </c>
       <c r="E47" s="17" t="n">
-        <f aca="false">(E12*Assumptions!$B$12+E13*Assumptions!$C$12+E14*Assumptions!$D$12)*12</f>
+        <f aca="false">(E12*Assumptions!$B$12+E13*Assumptions!$C$12+E14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>6000</v>
       </c>
       <c r="F47" s="17" t="n">
-        <f aca="false">(F12*Assumptions!$B$12+F13*Assumptions!$C$12+F14*Assumptions!$D$12)*12</f>
+        <f aca="false">(F12*Assumptions!$B$12+F13*Assumptions!$C$12+F14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>11947.5503342718</v>
       </c>
       <c r="G47" s="17" t="n">
-        <f aca="false">(G12*Assumptions!$B$12+G13*Assumptions!$C$12+G14*Assumptions!$D$12)*12</f>
+        <f aca="false">(G12*Assumptions!$B$12+G13*Assumptions!$C$12+G14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>17843.109497388</v>
       </c>
       <c r="H47" s="17" t="n">
-        <f aca="false">(H12*Assumptions!$B$12+H13*Assumptions!$C$12+H14*Assumptions!$D$12)*12</f>
+        <f aca="false">(H12*Assumptions!$B$12+H13*Assumptions!$C$12+H14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>39687.1319759397</v>
       </c>
       <c r="I47" s="17" t="n">
-        <f aca="false">(I12*Assumptions!$B$12+I13*Assumptions!$C$12+I14*Assumptions!$D$12)*12</f>
+        <f aca="false">(I12*Assumptions!$B$12+I13*Assumptions!$C$12+I14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>61340.2025082984</v>
       </c>
       <c r="J47" s="17" t="n">
-        <f aca="false">(J12*Assumptions!$B$12+J13*Assumptions!$C$12+J14*Assumptions!$D$12)*12</f>
+        <f aca="false">(J12*Assumptions!$B$12+J13*Assumptions!$C$12+J14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>82803.9903220885</v>
       </c>
       <c r="K47" s="17" t="n">
-        <f aca="false">(K12*Assumptions!$B$12+K13*Assumptions!$C$12+K14*Assumptions!$D$12)*12</f>
+        <f aca="false">(K12*Assumptions!$B$12+K13*Assumptions!$C$12+K14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>104080.150053196</v>
       </c>
       <c r="L47" s="17" t="n">
-        <f aca="false">(L12*Assumptions!$B$12+L13*Assumptions!$C$12+L14*Assumptions!$D$12)*12</f>
+        <f aca="false">(L12*Assumptions!$B$12+L13*Assumptions!$C$12+L14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>125170.321873325</v>
       </c>
       <c r="M47" s="17" t="n">
-        <f aca="false">(M12*Assumptions!$B$12+M13*Assumptions!$C$12+M14*Assumptions!$D$12)*12</f>
+        <f aca="false">(M12*Assumptions!$B$12+M13*Assumptions!$C$12+M14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>146076.131616434</v>
       </c>
       <c r="N47" s="17" t="n">
-        <f aca="false">(N12*Assumptions!$B$12+N13*Assumptions!$C$12+N14*Assumptions!$D$12)*12</f>
+        <f aca="false">(N12*Assumptions!$B$12+N13*Assumptions!$C$12+N14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>172799.190904076</v>
       </c>
       <c r="O47" s="17" t="n">
-        <f aca="false">(O12*Assumptions!$B$12+O13*Assumptions!$C$12+O14*Assumptions!$D$12)*12</f>
+        <f aca="false">(O12*Assumptions!$B$12+O13*Assumptions!$C$12+O14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>199288.647603906</v>
       </c>
       <c r="P47" s="17" t="n">
-        <f aca="false">(P12*Assumptions!$B$12+P13*Assumptions!$C$12+P14*Assumptions!$D$12)*12</f>
+        <f aca="false">(P12*Assumptions!$B$12+P13*Assumptions!$C$12+P14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>225546.543778865</v>
       </c>
       <c r="Q47" s="17" t="n">
-        <f aca="false">(Q12*Assumptions!$B$12+Q13*Assumptions!$C$12+Q14*Assumptions!$D$12)*12</f>
+        <f aca="false">(Q12*Assumptions!$B$12+Q13*Assumptions!$C$12+Q14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>267574.903640974</v>
       </c>
       <c r="R47" s="17" t="n">
-        <f aca="false">(R12*Assumptions!$B$12+R13*Assumptions!$C$12+R14*Assumptions!$D$12)*12</f>
+        <f aca="false">(R12*Assumptions!$B$12+R13*Assumptions!$C$12+R14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>309235.867932104</v>
       </c>
       <c r="S47" s="17" t="n">
-        <f aca="false">(S12*Assumptions!$B$12+S13*Assumptions!$C$12+S14*Assumptions!$D$12)*12</f>
+        <f aca="false">(S12*Assumptions!$B$12+S13*Assumptions!$C$12+S14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>350532.648281404</v>
       </c>
       <c r="T47" s="17" t="n">
-        <f aca="false">(T12*Assumptions!$B$12+T13*Assumptions!$C$12+T14*Assumptions!$D$12)*12</f>
+        <f aca="false">(T12*Assumptions!$B$12+T13*Assumptions!$C$12+T14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>425468.428243208</v>
       </c>
       <c r="U47" s="17" t="n">
-        <f aca="false">(U12*Assumptions!$B$12+U13*Assumptions!$C$12+U14*Assumptions!$D$12)*12</f>
+        <f aca="false">(U12*Assumptions!$B$12+U13*Assumptions!$C$12+U14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>499749.14877</v>
       </c>
       <c r="V47" s="17" t="n">
-        <f aca="false">(V12*Assumptions!$B$12+V13*Assumptions!$C$12+V14*Assumptions!$D$12)*12</f>
+        <f aca="false">(V12*Assumptions!$B$12+V13*Assumptions!$C$12+V14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>573380.536136512</v>
       </c>
       <c r="W47" s="17" t="n">
-        <f aca="false">(W12*Assumptions!$B$12+W13*Assumptions!$C$12+W14*Assumptions!$D$12)*12</f>
+        <f aca="false">(W12*Assumptions!$B$12+W13*Assumptions!$C$12+W14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>612368.266560611</v>
       </c>
       <c r="X47" s="17" t="n">
-        <f aca="false">(X12*Assumptions!$B$12+X13*Assumptions!$C$12+X14*Assumptions!$D$12)*12</f>
+        <f aca="false">(X12*Assumptions!$B$12+X13*Assumptions!$C$12+X14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>651015.181413336</v>
       </c>
       <c r="Y47" s="17" t="n">
-        <f aca="false">(Y12*Assumptions!$B$12+Y13*Assumptions!$C$12+Y14*Assumptions!$D$12)*12</f>
+        <f aca="false">(Y12*Assumptions!$B$12+Y13*Assumptions!$C$12+Y14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>689324.259971819</v>
       </c>
       <c r="Z47" s="17" t="n">
-        <f aca="false">(Z12*Assumptions!$B$12+Z13*Assumptions!$C$12+Z14*Assumptions!$D$12)*12</f>
+        <f aca="false">(Z12*Assumptions!$B$12+Z13*Assumptions!$C$12+Z14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>783298.455469511</v>
       </c>
       <c r="AA47" s="17" t="n">
-        <f aca="false">(AA12*Assumptions!$B$12+AA13*Assumptions!$C$12+AA14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AA12*Assumptions!$B$12+AA13*Assumptions!$C$12+AA14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>876451.165110382</v>
       </c>
       <c r="AB47" s="17" t="n">
-        <f aca="false">(AB12*Assumptions!$B$12+AB13*Assumptions!$C$12+AB14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AB12*Assumptions!$B$12+AB13*Assumptions!$C$12+AB14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>968789.570004197</v>
       </c>
       <c r="AC47" s="17" t="n">
-        <f aca="false">(AC12*Assumptions!$B$12+AC13*Assumptions!$C$12+AC14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AC12*Assumptions!$B$12+AC13*Assumptions!$C$12+AC14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1026320.78848625</v>
       </c>
       <c r="AD47" s="17" t="n">
-        <f aca="false">(AD12*Assumptions!$B$12+AD13*Assumptions!$C$12+AD14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AD12*Assumptions!$B$12+AD13*Assumptions!$C$12+AD14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1083349.09143859</v>
       </c>
       <c r="AE47" s="17" t="n">
-        <f aca="false">(AE12*Assumptions!$B$12+AE13*Assumptions!$C$12+AE14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AE12*Assumptions!$B$12+AE13*Assumptions!$C$12+AE14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1139878.87515311</v>
       </c>
       <c r="AF47" s="17" t="n">
-        <f aca="false">(AF12*Assumptions!$B$12+AF13*Assumptions!$C$12+AF14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AF12*Assumptions!$B$12+AF13*Assumptions!$C$12+AF14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1245914.49749104</v>
       </c>
       <c r="AG47" s="17" t="n">
-        <f aca="false">(AG12*Assumptions!$B$12+AG13*Assumptions!$C$12+AG14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AG12*Assumptions!$B$12+AG13*Assumptions!$C$12+AG14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1351023.19767116</v>
       </c>
       <c r="AH47" s="17" t="n">
-        <f aca="false">(AH12*Assumptions!$B$12+AH13*Assumptions!$C$12+AH14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AH12*Assumptions!$B$12+AH13*Assumptions!$C$12+AH14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1455213.07848635</v>
       </c>
       <c r="AI47" s="17" t="n">
-        <f aca="false">(AI12*Assumptions!$B$12+AI13*Assumptions!$C$12+AI14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AI12*Assumptions!$B$12+AI13*Assumptions!$C$12+AI14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1564492.17189803</v>
       </c>
       <c r="AJ47" s="17" t="n">
-        <f aca="false">(AJ12*Assumptions!$B$12+AJ13*Assumptions!$C$12+AJ14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AJ12*Assumptions!$B$12+AJ13*Assumptions!$C$12+AJ14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1672815.98998963</v>
       </c>
       <c r="AK47" s="17" t="n">
-        <f aca="false">(AK12*Assumptions!$B$12+AK13*Assumptions!$C$12+AK14*Assumptions!$D$12)*12</f>
+        <f aca="false">(AK12*Assumptions!$B$12+AK13*Assumptions!$C$12+AK14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
         <v>1780192.88340635</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B48" s="20" t="n">
         <f aca="false">IF(AND(B42&gt;=0,C48&lt;&gt;999),B$2,999)</f>
@@ -9497,7 +9539,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B49" s="20" t="n">
         <f aca="false">IF('Opex Plan'!$C$13&lt;=0,1,0)</f>
@@ -9646,7 +9688,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B50" s="20" t="n">
         <f aca="false">IF('Opex Plan'!$C$14&lt;=0,1,0)</f>
@@ -9795,7 +9837,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B51" s="20" t="n">
         <f aca="false">IF('Opex Plan'!$C$15&lt;=0,1,0)</f>
@@ -9944,7 +9986,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B52" s="20" t="n">
         <f aca="false">IF('Opex Plan'!$C$16&lt;=0,1,0)</f>
@@ -10118,17 +10160,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B4" s="30"/>
       <c r="C4" s="30"/>
@@ -10137,24 +10179,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="B6" s="23" t="n">
         <v>1</v>
@@ -10167,12 +10209,12 @@
         <v>4699</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B7" s="23" t="n">
         <v>1</v>
@@ -10185,12 +10227,12 @@
         <v>400</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="B8" s="23" t="n">
         <v>1</v>
@@ -10203,12 +10245,12 @@
         <v>250</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B9" s="23" t="n">
         <v>1</v>
@@ -10221,12 +10263,12 @@
         <v>150</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D10" s="33" t="n">
         <f aca="false">SUM(D6:D9)</f>
@@ -10235,12 +10277,12 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B13" s="30"/>
       <c r="C13" s="30"/>
@@ -10249,24 +10291,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B15" s="23" t="n">
         <v>1</v>
@@ -10279,12 +10321,12 @@
         <v>19628</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B16" s="23" t="n">
         <v>1</v>
@@ -10297,12 +10339,12 @@
         <v>650</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="B17" s="23" t="n">
         <v>1</v>
@@ -10315,12 +10357,12 @@
         <v>1100</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B18" s="23" t="n">
         <v>1</v>
@@ -10333,12 +10375,12 @@
         <v>700</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="B19" s="23" t="n">
         <v>1</v>
@@ -10351,12 +10393,12 @@
         <v>250</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D20" s="33" t="n">
         <f aca="false">SUM(D15:D19)</f>
@@ -10365,12 +10407,12 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="30"/>
@@ -10379,24 +10421,24 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="B25" s="23" t="n">
         <v>2</v>
@@ -10409,12 +10451,12 @@
         <v>34000</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="B26" s="23" t="n">
         <v>1</v>
@@ -10427,12 +10469,12 @@
         <v>20000</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B27" s="23" t="n">
         <v>1</v>
@@ -10445,12 +10487,12 @@
         <v>1800</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B28" s="23" t="n">
         <v>1</v>
@@ -10463,12 +10505,12 @@
         <v>1500</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B29" s="23" t="n">
         <v>1</v>
@@ -10481,12 +10523,12 @@
         <v>700</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="D30" s="33" t="n">
         <f aca="false">SUM(D25:D29)</f>
@@ -10495,7 +10537,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -10526,335 +10568,335 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>300</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>

</xml_diff>